<commit_message>
Update example test file RowSettings
Update reference test file for example RowSettings. After style
infrastructure switch, the styles part is saved differently. The test
file has been updated, no semantic change.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Rows/RowSettings.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Rows/RowSettings.xlsx
@@ -18,85 +18,64 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="4">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFF0000"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFF8C00"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="3">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="3">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="4">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8C00"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>